<commit_message>
feat: dynamic Excel import with GUI — File > Import Telemetry Definitions
- import_from_excel.py: unified import script supporting any sheet name
  as tm_type (first word, lowercased). Auto-generates telemetry YAML +
  enums.yaml with MSB->LSB conversion built in.
- main_window.py: added menu bar with '文件 > 导入遥测定义' action
  Opens QFileDialog, runs import, shows summary with copy instructions
- PLAN.md: updated M2 to document dynamic import capability
- get_available_tm_types() method added to NebulaRS422Protocol
  (provides future-proof scanning of product YAML files)
</commit_message>
<xml_diff>
--- a/项目文档/通讯协议/excel版遥测大表/PPCU_Telemetry_Database_v4.xlsx
+++ b/项目文档/通讯协议/excel版遥测大表/PPCU_Telemetry_Database_v4.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Codex Workspace\01_Projects\项目文档\通讯协议\excel版遥测大表\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{979FFD57-D570-40CC-9675-37D2A99B7AD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA13FC14-5DD5-4DD4-AE02-8BD40655D2EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TM1 参数表" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1400" uniqueCount="530">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1400" uniqueCount="531">
   <si>
     <t>序号</t>
   </si>
@@ -1622,13 +1622,45 @@
   </si>
   <si>
     <t>TM3105</t>
+  </si>
+  <si>
+    <r>
+      <t>0:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="微软雅黑"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>关</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>; 3:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="微软雅黑"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>开</t>
+    </r>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1666,6 +1698,12 @@
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="微软雅黑"/>
+      <family val="2"/>
+      <charset val="134"/>
     </font>
   </fonts>
   <fills count="4">
@@ -3320,7 +3358,7 @@
         <v>262</v>
       </c>
       <c r="N29" s="2" t="s">
-        <v>263</v>
+        <v>530</v>
       </c>
     </row>
     <row r="30" spans="1:19" ht="14.5" customHeight="1">
@@ -8336,7 +8374,9 @@
         <v>17</v>
       </c>
       <c r="I22" s="6"/>
-      <c r="J22" s="6"/>
+      <c r="J22" s="6">
+        <v>6</v>
+      </c>
       <c r="K22" s="6"/>
       <c r="L22" s="6"/>
       <c r="M22" s="6"/>
@@ -8368,7 +8408,9 @@
         <v>17</v>
       </c>
       <c r="I23" s="6"/>
-      <c r="J23" s="6"/>
+      <c r="J23" s="6">
+        <v>6</v>
+      </c>
       <c r="K23" s="6"/>
       <c r="L23" s="6"/>
       <c r="M23" s="6"/>
@@ -8400,7 +8442,9 @@
         <v>17</v>
       </c>
       <c r="I24" s="6"/>
-      <c r="J24" s="6"/>
+      <c r="J24" s="6">
+        <v>6</v>
+      </c>
       <c r="K24" s="6"/>
       <c r="L24" s="6"/>
       <c r="M24" s="6"/>
@@ -8432,7 +8476,9 @@
         <v>17</v>
       </c>
       <c r="I25" s="6"/>
-      <c r="J25" s="6"/>
+      <c r="J25" s="6">
+        <v>6</v>
+      </c>
       <c r="K25" s="6"/>
       <c r="L25" s="6"/>
       <c r="M25" s="6"/>
@@ -8464,7 +8510,9 @@
         <v>17</v>
       </c>
       <c r="I26" s="6"/>
-      <c r="J26" s="6"/>
+      <c r="J26" s="6">
+        <v>6</v>
+      </c>
       <c r="K26" s="6"/>
       <c r="L26" s="6"/>
       <c r="M26" s="6"/>
@@ -8496,7 +8544,9 @@
         <v>17</v>
       </c>
       <c r="I27" s="6"/>
-      <c r="J27" s="6"/>
+      <c r="J27" s="6">
+        <v>6</v>
+      </c>
       <c r="K27" s="6"/>
       <c r="L27" s="6"/>
       <c r="M27" s="6"/>
@@ -8528,7 +8578,9 @@
         <v>17</v>
       </c>
       <c r="I28" s="6"/>
-      <c r="J28" s="6"/>
+      <c r="J28" s="6">
+        <v>6</v>
+      </c>
       <c r="K28" s="6"/>
       <c r="L28" s="6"/>
       <c r="M28" s="6"/>
@@ -8560,7 +8612,9 @@
         <v>17</v>
       </c>
       <c r="I29" s="6"/>
-      <c r="J29" s="6"/>
+      <c r="J29" s="6">
+        <v>6</v>
+      </c>
       <c r="K29" s="6"/>
       <c r="L29" s="6"/>
       <c r="M29" s="6"/>
@@ -8592,7 +8646,9 @@
         <v>17</v>
       </c>
       <c r="I30" s="6"/>
-      <c r="J30" s="6"/>
+      <c r="J30" s="6">
+        <v>6</v>
+      </c>
       <c r="K30" s="6"/>
       <c r="L30" s="6"/>
       <c r="M30" s="6">
@@ -8626,7 +8682,9 @@
         <v>17</v>
       </c>
       <c r="I31" s="6"/>
-      <c r="J31" s="6"/>
+      <c r="J31" s="6">
+        <v>6</v>
+      </c>
       <c r="K31" s="6"/>
       <c r="L31" s="6"/>
       <c r="M31" s="6"/>
@@ -8658,7 +8716,9 @@
         <v>17</v>
       </c>
       <c r="I32" s="6"/>
-      <c r="J32" s="6"/>
+      <c r="J32" s="6">
+        <v>6</v>
+      </c>
       <c r="K32" s="6"/>
       <c r="L32" s="6"/>
       <c r="M32" s="6">
@@ -8692,7 +8752,9 @@
         <v>17</v>
       </c>
       <c r="I33" s="6"/>
-      <c r="J33" s="6"/>
+      <c r="J33" s="6">
+        <v>6</v>
+      </c>
       <c r="K33" s="6"/>
       <c r="L33" s="6"/>
       <c r="M33" s="6">
@@ -8726,7 +8788,9 @@
         <v>17</v>
       </c>
       <c r="I34" s="6"/>
-      <c r="J34" s="6"/>
+      <c r="J34" s="6">
+        <v>6</v>
+      </c>
       <c r="K34" s="6"/>
       <c r="L34" s="6"/>
       <c r="M34" s="6">
@@ -8760,7 +8824,9 @@
         <v>17</v>
       </c>
       <c r="I35" s="6"/>
-      <c r="J35" s="6"/>
+      <c r="J35" s="6">
+        <v>6</v>
+      </c>
       <c r="K35" s="6"/>
       <c r="L35" s="6"/>
       <c r="M35" s="6">
@@ -8794,7 +8860,9 @@
         <v>17</v>
       </c>
       <c r="I36" s="6"/>
-      <c r="J36" s="6"/>
+      <c r="J36" s="6">
+        <v>6</v>
+      </c>
       <c r="K36" s="6"/>
       <c r="L36" s="6"/>
       <c r="M36" s="6">
@@ -8828,7 +8896,9 @@
         <v>17</v>
       </c>
       <c r="I37" s="6"/>
-      <c r="J37" s="6"/>
+      <c r="J37" s="6">
+        <v>6</v>
+      </c>
       <c r="K37" s="6"/>
       <c r="L37" s="6"/>
       <c r="M37" s="6">
@@ -8862,7 +8932,9 @@
         <v>17</v>
       </c>
       <c r="I38" s="6"/>
-      <c r="J38" s="6"/>
+      <c r="J38" s="6">
+        <v>6</v>
+      </c>
       <c r="K38" s="6"/>
       <c r="L38" s="6"/>
       <c r="M38" s="6">
@@ -8896,7 +8968,9 @@
         <v>17</v>
       </c>
       <c r="I39" s="6"/>
-      <c r="J39" s="6"/>
+      <c r="J39" s="6">
+        <v>6</v>
+      </c>
       <c r="K39" s="6"/>
       <c r="L39" s="6"/>
       <c r="M39" s="6">
@@ -8930,7 +9004,9 @@
         <v>17</v>
       </c>
       <c r="I40" s="6"/>
-      <c r="J40" s="6"/>
+      <c r="J40" s="6">
+        <v>6</v>
+      </c>
       <c r="K40" s="6"/>
       <c r="L40" s="6"/>
       <c r="M40" s="6">
@@ -8964,7 +9040,9 @@
         <v>17</v>
       </c>
       <c r="I41" s="6"/>
-      <c r="J41" s="6"/>
+      <c r="J41" s="6">
+        <v>6</v>
+      </c>
       <c r="K41" s="6"/>
       <c r="L41" s="6"/>
       <c r="M41" s="6"/>
@@ -8996,7 +9074,9 @@
         <v>17</v>
       </c>
       <c r="I42" s="6"/>
-      <c r="J42" s="6"/>
+      <c r="J42" s="6">
+        <v>6</v>
+      </c>
       <c r="K42" s="6"/>
       <c r="L42" s="6"/>
       <c r="M42" s="6"/>
@@ -9028,7 +9108,9 @@
         <v>17</v>
       </c>
       <c r="I43" s="6"/>
-      <c r="J43" s="6"/>
+      <c r="J43" s="6">
+        <v>6</v>
+      </c>
       <c r="K43" s="6"/>
       <c r="L43" s="6"/>
       <c r="M43" s="6"/>
@@ -9060,7 +9142,9 @@
         <v>17</v>
       </c>
       <c r="I44" s="6"/>
-      <c r="J44" s="6"/>
+      <c r="J44" s="6">
+        <v>6</v>
+      </c>
       <c r="K44" s="6"/>
       <c r="L44" s="6"/>
       <c r="M44" s="6"/>
@@ -9092,7 +9176,9 @@
         <v>17</v>
       </c>
       <c r="I45" s="6"/>
-      <c r="J45" s="6"/>
+      <c r="J45" s="6">
+        <v>6</v>
+      </c>
       <c r="K45" s="6"/>
       <c r="L45" s="6"/>
       <c r="M45" s="6"/>
@@ -9124,7 +9210,9 @@
         <v>17</v>
       </c>
       <c r="I46" s="6"/>
-      <c r="J46" s="6"/>
+      <c r="J46" s="6">
+        <v>6</v>
+      </c>
       <c r="K46" s="6"/>
       <c r="L46" s="6"/>
       <c r="M46" s="6"/>
@@ -9156,7 +9244,9 @@
         <v>17</v>
       </c>
       <c r="I47" s="6"/>
-      <c r="J47" s="6"/>
+      <c r="J47" s="6">
+        <v>6</v>
+      </c>
       <c r="K47" s="6"/>
       <c r="L47" s="6"/>
       <c r="M47" s="6"/>
@@ -9188,7 +9278,9 @@
         <v>17</v>
       </c>
       <c r="I48" s="6"/>
-      <c r="J48" s="6"/>
+      <c r="J48" s="6">
+        <v>6</v>
+      </c>
       <c r="K48" s="6"/>
       <c r="L48" s="6"/>
       <c r="M48" s="6"/>
@@ -9220,7 +9312,9 @@
         <v>17</v>
       </c>
       <c r="I49" s="6"/>
-      <c r="J49" s="6"/>
+      <c r="J49" s="6">
+        <v>6</v>
+      </c>
       <c r="K49" s="6"/>
       <c r="L49" s="6"/>
       <c r="M49" s="6"/>
@@ -9252,7 +9346,9 @@
         <v>17</v>
       </c>
       <c r="I50" s="6"/>
-      <c r="J50" s="6"/>
+      <c r="J50" s="6">
+        <v>6</v>
+      </c>
       <c r="K50" s="6"/>
       <c r="L50" s="6"/>
       <c r="M50" s="6"/>
@@ -9284,7 +9380,9 @@
         <v>17</v>
       </c>
       <c r="I51" s="6"/>
-      <c r="J51" s="6"/>
+      <c r="J51" s="6">
+        <v>6</v>
+      </c>
       <c r="K51" s="6"/>
       <c r="L51" s="6"/>
       <c r="M51" s="6"/>
@@ -9316,7 +9414,9 @@
         <v>17</v>
       </c>
       <c r="I52" s="6"/>
-      <c r="J52" s="6"/>
+      <c r="J52" s="6">
+        <v>6</v>
+      </c>
       <c r="K52" s="6"/>
       <c r="L52" s="6"/>
       <c r="M52" s="6"/>
@@ -9348,7 +9448,9 @@
         <v>17</v>
       </c>
       <c r="I53" s="6"/>
-      <c r="J53" s="6"/>
+      <c r="J53" s="6">
+        <v>6</v>
+      </c>
       <c r="K53" s="6"/>
       <c r="L53" s="6"/>
       <c r="M53" s="6"/>
@@ -9380,7 +9482,9 @@
         <v>17</v>
       </c>
       <c r="I54" s="6"/>
-      <c r="J54" s="6"/>
+      <c r="J54" s="6">
+        <v>6</v>
+      </c>
       <c r="K54" s="6"/>
       <c r="L54" s="6"/>
       <c r="M54" s="6"/>
@@ -9412,7 +9516,9 @@
         <v>17</v>
       </c>
       <c r="I55" s="6"/>
-      <c r="J55" s="6"/>
+      <c r="J55" s="6">
+        <v>6</v>
+      </c>
       <c r="K55" s="6"/>
       <c r="L55" s="6"/>
       <c r="M55" s="6"/>
@@ -9444,7 +9550,9 @@
         <v>17</v>
       </c>
       <c r="I56" s="6"/>
-      <c r="J56" s="6"/>
+      <c r="J56" s="6">
+        <v>6</v>
+      </c>
       <c r="K56" s="6"/>
       <c r="L56" s="6"/>
       <c r="M56" s="6"/>
@@ -9476,7 +9584,9 @@
         <v>17</v>
       </c>
       <c r="I57" s="6"/>
-      <c r="J57" s="6"/>
+      <c r="J57" s="6">
+        <v>6</v>
+      </c>
       <c r="K57" s="6"/>
       <c r="L57" s="6"/>
       <c r="M57" s="6"/>
@@ -9508,7 +9618,9 @@
         <v>17</v>
       </c>
       <c r="I58" s="6"/>
-      <c r="J58" s="6"/>
+      <c r="J58" s="6">
+        <v>6</v>
+      </c>
       <c r="K58" s="6"/>
       <c r="L58" s="6"/>
       <c r="M58" s="6"/>
@@ -9540,7 +9652,9 @@
         <v>17</v>
       </c>
       <c r="I59" s="6"/>
-      <c r="J59" s="6"/>
+      <c r="J59" s="6">
+        <v>6</v>
+      </c>
       <c r="K59" s="6"/>
       <c r="L59" s="6"/>
       <c r="M59" s="6"/>
@@ -9572,7 +9686,9 @@
         <v>17</v>
       </c>
       <c r="I60" s="6"/>
-      <c r="J60" s="6"/>
+      <c r="J60" s="6">
+        <v>6</v>
+      </c>
       <c r="K60" s="6"/>
       <c r="L60" s="6"/>
       <c r="M60" s="6"/>
@@ -9604,7 +9720,9 @@
         <v>17</v>
       </c>
       <c r="I61" s="6"/>
-      <c r="J61" s="6"/>
+      <c r="J61" s="6">
+        <v>6</v>
+      </c>
       <c r="K61" s="6"/>
       <c r="L61" s="6"/>
       <c r="M61" s="6">
@@ -9638,7 +9756,9 @@
         <v>17</v>
       </c>
       <c r="I62" s="6"/>
-      <c r="J62" s="6"/>
+      <c r="J62" s="6">
+        <v>6</v>
+      </c>
       <c r="K62" s="6"/>
       <c r="L62" s="6"/>
       <c r="M62" s="6">
@@ -9672,7 +9792,9 @@
         <v>17</v>
       </c>
       <c r="I63" s="6"/>
-      <c r="J63" s="6"/>
+      <c r="J63" s="6">
+        <v>6</v>
+      </c>
       <c r="K63" s="6"/>
       <c r="L63" s="6"/>
       <c r="M63" s="6">
@@ -9706,7 +9828,9 @@
         <v>17</v>
       </c>
       <c r="I64" s="6"/>
-      <c r="J64" s="6"/>
+      <c r="J64" s="6">
+        <v>6</v>
+      </c>
       <c r="K64" s="6"/>
       <c r="L64" s="6"/>
       <c r="M64" s="6">
@@ -9740,7 +9864,9 @@
         <v>17</v>
       </c>
       <c r="I65" s="6"/>
-      <c r="J65" s="6"/>
+      <c r="J65" s="6">
+        <v>6</v>
+      </c>
       <c r="K65" s="6"/>
       <c r="L65" s="6"/>
       <c r="M65" s="6"/>
@@ -9772,7 +9898,9 @@
         <v>17</v>
       </c>
       <c r="I66" s="6"/>
-      <c r="J66" s="6"/>
+      <c r="J66" s="6">
+        <v>6</v>
+      </c>
       <c r="K66" s="6"/>
       <c r="L66" s="6"/>
       <c r="M66" s="6">
@@ -9806,7 +9934,9 @@
         <v>17</v>
       </c>
       <c r="I67" s="6"/>
-      <c r="J67" s="6"/>
+      <c r="J67" s="6">
+        <v>6</v>
+      </c>
       <c r="K67" s="6"/>
       <c r="L67" s="6"/>
       <c r="M67" s="6"/>
@@ -9838,7 +9968,9 @@
         <v>17</v>
       </c>
       <c r="I68" s="6"/>
-      <c r="J68" s="6"/>
+      <c r="J68" s="6">
+        <v>6</v>
+      </c>
       <c r="K68" s="6"/>
       <c r="L68" s="6"/>
       <c r="M68" s="6">
@@ -9872,7 +10004,9 @@
         <v>17</v>
       </c>
       <c r="I69" s="6"/>
-      <c r="J69" s="6"/>
+      <c r="J69" s="6">
+        <v>6</v>
+      </c>
       <c r="K69" s="6"/>
       <c r="L69" s="6"/>
       <c r="M69" s="6"/>
@@ -9904,7 +10038,9 @@
         <v>17</v>
       </c>
       <c r="I70" s="6"/>
-      <c r="J70" s="6"/>
+      <c r="J70" s="6">
+        <v>6</v>
+      </c>
       <c r="K70" s="6"/>
       <c r="L70" s="6"/>
       <c r="M70" s="6"/>
@@ -9936,7 +10072,9 @@
         <v>17</v>
       </c>
       <c r="I71" s="6"/>
-      <c r="J71" s="6"/>
+      <c r="J71" s="6">
+        <v>6</v>
+      </c>
       <c r="K71" s="6"/>
       <c r="L71" s="6"/>
       <c r="M71" s="6"/>
@@ -9968,7 +10106,9 @@
         <v>17</v>
       </c>
       <c r="I72" s="6"/>
-      <c r="J72" s="6"/>
+      <c r="J72" s="6">
+        <v>6</v>
+      </c>
       <c r="K72" s="6"/>
       <c r="L72" s="6"/>
       <c r="M72" s="6">
@@ -10002,7 +10142,9 @@
         <v>17</v>
       </c>
       <c r="I73" s="6"/>
-      <c r="J73" s="6"/>
+      <c r="J73" s="6">
+        <v>6</v>
+      </c>
       <c r="K73" s="6" t="s">
         <v>465</v>
       </c>
@@ -10036,7 +10178,9 @@
         <v>17</v>
       </c>
       <c r="I74" s="6"/>
-      <c r="J74" s="6"/>
+      <c r="J74" s="6">
+        <v>6</v>
+      </c>
       <c r="K74" s="6" t="s">
         <v>236</v>
       </c>
@@ -10070,7 +10214,9 @@
         <v>17</v>
       </c>
       <c r="I75" s="6"/>
-      <c r="J75" s="6"/>
+      <c r="J75" s="6">
+        <v>6</v>
+      </c>
       <c r="K75" s="6" t="s">
         <v>65</v>
       </c>
@@ -10104,7 +10250,9 @@
         <v>17</v>
       </c>
       <c r="I76" s="6"/>
-      <c r="J76" s="6"/>
+      <c r="J76" s="6">
+        <v>6</v>
+      </c>
       <c r="K76" s="6" t="s">
         <v>240</v>
       </c>
@@ -10140,7 +10288,9 @@
         <v>17</v>
       </c>
       <c r="I77" s="6"/>
-      <c r="J77" s="6"/>
+      <c r="J77" s="6">
+        <v>6</v>
+      </c>
       <c r="K77" s="6" t="s">
         <v>240</v>
       </c>
@@ -10176,7 +10326,9 @@
         <v>17</v>
       </c>
       <c r="I78" s="6"/>
-      <c r="J78" s="6"/>
+      <c r="J78" s="6">
+        <v>6</v>
+      </c>
       <c r="K78" s="6" t="s">
         <v>240</v>
       </c>
@@ -10212,7 +10364,9 @@
         <v>17</v>
       </c>
       <c r="I79" s="6"/>
-      <c r="J79" s="6"/>
+      <c r="J79" s="6">
+        <v>6</v>
+      </c>
       <c r="K79" s="6" t="s">
         <v>240</v>
       </c>
@@ -10248,7 +10402,9 @@
         <v>17</v>
       </c>
       <c r="I80" s="6"/>
-      <c r="J80" s="6"/>
+      <c r="J80" s="6">
+        <v>6</v>
+      </c>
       <c r="K80" s="6" t="s">
         <v>240</v>
       </c>
@@ -10284,7 +10440,9 @@
         <v>17</v>
       </c>
       <c r="I81" s="6"/>
-      <c r="J81" s="6"/>
+      <c r="J81" s="6">
+        <v>6</v>
+      </c>
       <c r="K81" s="6" t="s">
         <v>240</v>
       </c>
@@ -10320,7 +10478,9 @@
         <v>17</v>
       </c>
       <c r="I82" s="6"/>
-      <c r="J82" s="6"/>
+      <c r="J82" s="6">
+        <v>6</v>
+      </c>
       <c r="K82" s="6" t="s">
         <v>240</v>
       </c>
@@ -10356,7 +10516,9 @@
         <v>17</v>
       </c>
       <c r="I83" s="6"/>
-      <c r="J83" s="6"/>
+      <c r="J83" s="6">
+        <v>6</v>
+      </c>
       <c r="K83" s="6" t="s">
         <v>240</v>
       </c>
@@ -10392,7 +10554,9 @@
         <v>17</v>
       </c>
       <c r="I84" s="6"/>
-      <c r="J84" s="6"/>
+      <c r="J84" s="6">
+        <v>6</v>
+      </c>
       <c r="K84" s="6" t="s">
         <v>236</v>
       </c>
@@ -10426,7 +10590,9 @@
         <v>17</v>
       </c>
       <c r="I85" s="6"/>
-      <c r="J85" s="6"/>
+      <c r="J85" s="6">
+        <v>6</v>
+      </c>
       <c r="K85" s="6" t="s">
         <v>236</v>
       </c>
@@ -10460,7 +10626,9 @@
         <v>17</v>
       </c>
       <c r="I86" s="6"/>
-      <c r="J86" s="6"/>
+      <c r="J86" s="6">
+        <v>6</v>
+      </c>
       <c r="K86" s="6" t="s">
         <v>240</v>
       </c>
@@ -10496,7 +10664,9 @@
         <v>17</v>
       </c>
       <c r="I87" s="6"/>
-      <c r="J87" s="6"/>
+      <c r="J87" s="6">
+        <v>6</v>
+      </c>
       <c r="K87" s="6" t="s">
         <v>65</v>
       </c>
@@ -10530,7 +10700,9 @@
         <v>17</v>
       </c>
       <c r="I88" s="6"/>
-      <c r="J88" s="6"/>
+      <c r="J88" s="6">
+        <v>6</v>
+      </c>
       <c r="K88" s="6" t="s">
         <v>36</v>
       </c>
@@ -10566,7 +10738,9 @@
         <v>17</v>
       </c>
       <c r="I89" s="6"/>
-      <c r="J89" s="6"/>
+      <c r="J89" s="6">
+        <v>6</v>
+      </c>
       <c r="K89" s="6" t="s">
         <v>36</v>
       </c>
@@ -10602,7 +10776,9 @@
         <v>17</v>
       </c>
       <c r="I90" s="6"/>
-      <c r="J90" s="6"/>
+      <c r="J90" s="6">
+        <v>6</v>
+      </c>
       <c r="K90" s="6" t="s">
         <v>240</v>
       </c>
@@ -10638,7 +10814,9 @@
         <v>17</v>
       </c>
       <c r="I91" s="6"/>
-      <c r="J91" s="6"/>
+      <c r="J91" s="6">
+        <v>6</v>
+      </c>
       <c r="K91" s="6" t="s">
         <v>65</v>
       </c>
@@ -10672,7 +10850,9 @@
         <v>17</v>
       </c>
       <c r="I92" s="6"/>
-      <c r="J92" s="6"/>
+      <c r="J92" s="6">
+        <v>6</v>
+      </c>
       <c r="K92" s="6" t="s">
         <v>65</v>
       </c>
@@ -10708,7 +10888,9 @@
         <v>17</v>
       </c>
       <c r="I93" s="6"/>
-      <c r="J93" s="6"/>
+      <c r="J93" s="6">
+        <v>6</v>
+      </c>
       <c r="K93" s="6" t="s">
         <v>65</v>
       </c>

</xml_diff>